<commit_message>
Update: - Fixing import leasing
</commit_message>
<xml_diff>
--- a/x_leasing_amortization/static/templates/Template_Import_Leasing.xlsx
+++ b/x_leasing_amortization/static/templates/Template_Import_Leasing.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Header" sheetId="1" r:id="R4967e7b466624dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angsuran" sheetId="2" r:id="R1e30d71ebdd74906"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="3" r:id="Rfe7486ea869442c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Header" sheetId="1" r:id="R156f3d51abc549e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angsuran" sheetId="2" r:id="R823682a3914444d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="3" r:id="R312f576edd55424b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1263,7 +1263,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>Hasil impor tetap Draft, belum ada pembayaran/jurnal. Review lalu Confirm di Odoo.</x:v>
+        <x:v>Hasil impor tetap Draft tanpa pembayaran/jurnal. Lengkapi Vehicle dan Analytic Account sebelum Confirm.</x:v>
       </x:c>
       <x:c r="C11" s="1"/>
       <x:c r="D11" s="1"/>
@@ -1323,7 +1323,7 @@
         <x:v>Referensi</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
-        <x:v>Vendor: nama persis. Plate Number: nopol persis. Account: kode CoA persis. Interest Journal: kode jurnal umum persis.</x:v>
+        <x:v>Vendor: nama persis. Account: kode CoA persis. Interest Journal: kode jurnal umum persis. Plate Number opsional.</x:v>
       </x:c>
       <x:c r="C17" s="1"/>
       <x:c r="D17" s="1"/>
@@ -1333,7 +1333,7 @@
         <x:v>Referensi ambigu</x:v>
       </x:c>
       <x:c r="B18" s="17" t="str">
-        <x:v>Nama vendor/nopol/kode harus unik pada company. Impor tidak membuat vendor, kendaraan, akun atau jurnal baru.</x:v>
+        <x:v>Nopol tidak cocok/tidak unik disimpan sebagai teks tanpa link Vehicle. Impor tidak membuat master data baru.</x:v>
       </x:c>
       <x:c r="C18" s="1"/>
       <x:c r="D18" s="1"/>
@@ -1343,7 +1343,7 @@
         <x:v>Tanpa PO</x:v>
       </x:c>
       <x:c r="B19" s="17" t="str">
-        <x:v>Impor membuat kontrak mandiri tanpa link ke PO. Agreement No. dan Leasing Contract No. diambil dari file.</x:v>
+        <x:v>Tanpa link PO. Agreement No., Leasing Contract No. dan Plate Number boleh kosong atau sama pada Import Key berbeda.</x:v>
       </x:c>
       <x:c r="C19" s="1"/>
       <x:c r="D19" s="1"/>
@@ -1483,7 +1483,7 @@
         <x:v>Agreement No.</x:v>
       </x:c>
       <x:c r="B34" s="17" t="str">
-        <x:v>Wajib, nomor agreement kontrak leasing.</x:v>
+        <x:v>Opsional, nomor agreement dari file. Tidak diperiksa keunikan atau kecocokannya dengan data lama.</x:v>
       </x:c>
       <x:c r="C34" s="1"/>
       <x:c r="D34" s="1"/>
@@ -1493,7 +1493,7 @@
         <x:v>Leasing Contract No.</x:v>
       </x:c>
       <x:c r="B35" s="17" t="str">
-        <x:v>Opsional, nomor kontrak leasing tambahan.</x:v>
+        <x:v>Opsional, nomor kontrak dari file. Boleh kosong atau sama pada kontrak lain.</x:v>
       </x:c>
       <x:c r="C35" s="1"/>
       <x:c r="D35" s="1"/>
@@ -1513,7 +1513,7 @@
         <x:v>Plate Number</x:v>
       </x:c>
       <x:c r="B37" s="17" t="str">
-        <x:v>Wajib, nopol kendaraan di company ini; kendaraan sudah memiliki analytic account.</x:v>
+        <x:v>Opsional, nopol dari file. Link Vehicle hanya jika ditemukan satu kendaraan pada company yang dipilih.</x:v>
       </x:c>
       <x:c r="C37" s="1"/>
       <x:c r="D37" s="1"/>

</xml_diff>